<commit_message>
Update East Passyunk vacancy classifications and add seasonal closure state
- Correct 13 EPA parcel classifications from source
- 1646, 1716, 1830, 1912 reclassified active
- Add distinct seasonal_closure map state with amber color, filter, legend, popup, and block stats
- 1637 and 1639 now render as seasonal closure rather than long-term
- Regenerate parcels.geojson via no-geocode rebuild

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/south-street-fieldwork-data.xlsx
+++ b/public/data/south-street-fieldwork-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brand\south-street-site\source-files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brand\south-street-site\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5214D1C6-F076-4FEA-B404-24601E9EB737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758C38B5-C110-4E3D-A6F9-E759767CFF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33720" yWindow="3300" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building Level Data" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7197" uniqueCount="1848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7202" uniqueCount="1849">
   <si>
     <t>Structural</t>
   </si>
@@ -5606,6 +5606,9 @@
   </si>
   <si>
     <t>Laff House</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -41885,7 +41888,7 @@
         <v>58</v>
       </c>
       <c r="Y316" s="21" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="Z316" s="21" t="str">
         <f>IF(U316="Vacant","Vacant","")</f>
@@ -43550,32 +43553,30 @@
       <c r="S331" s="14"/>
       <c r="T331" s="14"/>
       <c r="U331" s="21" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="V331" s="21">
         <f>IF(U331="",0,VLOOKUP(U331,Dropdown_Lists!$B$2:$C$31,2,FALSE))</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W331" s="21" t="str">
         <f>IF(U331="","",VLOOKUP(U331,Dropdown_Lists!$B$2:$D$31,3,FALSE))</f>
-        <v>Vacant</v>
+        <v>Food &amp; Drink</v>
       </c>
       <c r="X331" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y331" s="21" t="s">
-        <v>63</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="Y331" s="21"/>
       <c r="Z331" s="21" t="str">
         <f>IF(U331="Vacant","Vacant","")</f>
-        <v>Vacant</v>
+        <v/>
       </c>
       <c r="AA331" s="21" t="s">
         <v>44</v>
       </c>
       <c r="AB331" s="21" t="str">
         <f t="shared" si="19"/>
-        <v>Vacant</v>
+        <v/>
       </c>
       <c r="AC331" s="21">
         <v>2</v>
@@ -43583,17 +43584,14 @@
       <c r="AD331" s="21">
         <v>3</v>
       </c>
-      <c r="AE331" s="21" t="str">
-        <f>IF(U331="Vacant","","")</f>
-        <v/>
-      </c>
-      <c r="AF331" s="21" t="str">
-        <f>IF(U331="Vacant","No","")</f>
-        <v>No</v>
-      </c>
-      <c r="AG331" s="21" t="str">
-        <f>IF(U331="Vacant","6 N/A","")</f>
-        <v>6 N/A</v>
+      <c r="AE331" s="21">
+        <v>4</v>
+      </c>
+      <c r="AF331" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG331" s="21">
+        <v>4</v>
       </c>
       <c r="AH331" t="s">
         <v>1110</v>
@@ -43683,7 +43681,7 @@
         <v>58</v>
       </c>
       <c r="Y332" s="21" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="Z332" s="21" t="str">
         <f>IF(U332="Vacant","Vacant","")</f>
@@ -44462,32 +44460,29 @@
       <c r="S339" s="14"/>
       <c r="T339" s="14"/>
       <c r="U339" s="21" t="s">
-        <v>25</v>
+        <v>444</v>
       </c>
       <c r="V339" s="21">
         <f>IF(U339="",0,VLOOKUP(U339,Dropdown_Lists!$B$2:$C$31,2,FALSE))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="W339" s="21" t="str">
         <f>IF(U339="","",VLOOKUP(U339,Dropdown_Lists!$B$2:$D$31,3,FALSE))</f>
-        <v>Vacant</v>
+        <v>Professional Services</v>
       </c>
       <c r="X339" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y339" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z339" s="21" t="str">
-        <f>IF(U339="Vacant","Vacant","")</f>
-        <v>Vacant</v>
+        <v>44</v>
+      </c>
+      <c r="Y339" s="21"/>
+      <c r="Z339" s="21" t="s">
+        <v>54</v>
       </c>
       <c r="AA339" s="21" t="s">
         <v>44</v>
       </c>
       <c r="AB339" s="21" t="str">
         <f t="shared" si="19"/>
-        <v>Vacant</v>
+        <v/>
       </c>
       <c r="AC339" s="21">
         <v>4</v>
@@ -44495,17 +44490,14 @@
       <c r="AD339" s="21">
         <v>4</v>
       </c>
-      <c r="AE339" s="21" t="str">
-        <f>IF(U339="Vacant","","")</f>
-        <v/>
-      </c>
-      <c r="AF339" s="21" t="str">
-        <f>IF(U339="Vacant","No","")</f>
-        <v>No</v>
-      </c>
-      <c r="AG339" s="21" t="str">
-        <f>IF(U339="Vacant","6 N/A","")</f>
-        <v>6 N/A</v>
+      <c r="AE339" s="21">
+        <v>4</v>
+      </c>
+      <c r="AF339" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG339" s="21">
+        <v>2</v>
       </c>
       <c r="AH339" t="s">
         <v>1135</v>
@@ -47066,7 +47058,7 @@
         <v>58</v>
       </c>
       <c r="Y362" s="21" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Z362" s="21" t="str">
         <f>IF(U362="Vacant","Vacant","")</f>
@@ -47623,32 +47615,31 @@
       <c r="S367" s="14"/>
       <c r="T367" s="14"/>
       <c r="U367" s="21" t="s">
-        <v>25</v>
+        <v>444</v>
       </c>
       <c r="V367" s="21">
         <f>IF(U367="",0,VLOOKUP(U367,Dropdown_Lists!$B$2:$C$31,2,FALSE))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="W367" s="21" t="str">
         <f>IF(U367="","",VLOOKUP(U367,Dropdown_Lists!$B$2:$D$31,3,FALSE))</f>
-        <v>Vacant</v>
+        <v>Professional Services</v>
       </c>
       <c r="X367" s="21" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="Y367" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z367" s="21" t="str">
-        <f>IF(U367="Vacant","Vacant","")</f>
-        <v>Vacant</v>
+        <v>1848</v>
+      </c>
+      <c r="Z367" s="21" t="s">
+        <v>332</v>
       </c>
       <c r="AA367" s="21" t="s">
         <v>44</v>
       </c>
       <c r="AB367" s="21" t="str">
         <f t="shared" si="20"/>
-        <v>Vacant</v>
+        <v/>
       </c>
       <c r="AC367" s="21">
         <v>4</v>
@@ -47656,17 +47647,14 @@
       <c r="AD367" s="21">
         <v>5</v>
       </c>
-      <c r="AE367" s="21" t="str">
-        <f>IF(U367="Vacant","","")</f>
-        <v/>
-      </c>
-      <c r="AF367" s="21" t="str">
-        <f>IF(U367="Vacant","No","")</f>
-        <v>No</v>
-      </c>
-      <c r="AG367" s="21" t="str">
-        <f>IF(U367="Vacant","6 N/A","")</f>
-        <v>6 N/A</v>
+      <c r="AE367" s="21">
+        <v>3</v>
+      </c>
+      <c r="AF367" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG367" s="21">
+        <v>2</v>
       </c>
       <c r="AH367" t="s">
         <v>1218</v>
@@ -48874,7 +48862,7 @@
         <v>58</v>
       </c>
       <c r="Y378" s="21" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="Z378" s="21" t="str">
         <f>IF(U378="Vacant","Vacant","")</f>
@@ -49090,32 +49078,31 @@
       <c r="S380" s="14"/>
       <c r="T380" s="14"/>
       <c r="U380" s="21" t="s">
-        <v>25</v>
+        <v>405</v>
       </c>
       <c r="V380" s="21">
         <f>IF(U380="",0,VLOOKUP(U380,Dropdown_Lists!$B$2:$C$31,2,FALSE))</f>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="W380" s="21" t="str">
         <f>IF(U380="","",VLOOKUP(U380,Dropdown_Lists!$B$2:$D$31,3,FALSE))</f>
-        <v>Vacant</v>
+        <v>Retail Goods</v>
       </c>
       <c r="X380" s="21" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="Y380" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z380" s="21" t="str">
-        <f>IF(U380="Vacant","Vacant","")</f>
-        <v>Vacant</v>
+        <v>1848</v>
+      </c>
+      <c r="Z380" s="21" t="s">
+        <v>54</v>
       </c>
       <c r="AA380" s="21" t="s">
         <v>44</v>
       </c>
       <c r="AB380" s="21" t="str">
         <f t="shared" si="21"/>
-        <v>Vacant</v>
+        <v/>
       </c>
       <c r="AC380" s="21">
         <v>5</v>
@@ -49123,17 +49110,14 @@
       <c r="AD380" s="21">
         <v>5</v>
       </c>
-      <c r="AE380" s="21" t="str">
-        <f>IF(U380="Vacant","","")</f>
-        <v/>
-      </c>
-      <c r="AF380" s="21" t="str">
-        <f>IF(U380="Vacant","No","")</f>
-        <v>No</v>
-      </c>
-      <c r="AG380" s="21" t="str">
-        <f>IF(U380="Vacant","6 N/A","")</f>
-        <v>6 N/A</v>
+      <c r="AE380" s="21">
+        <v>2</v>
+      </c>
+      <c r="AF380" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG380" s="21">
+        <v>3</v>
       </c>
       <c r="AH380" t="s">
         <v>1255</v>
@@ -56329,7 +56313,7 @@
         <v>58</v>
       </c>
       <c r="Y446" s="21" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="Z446" s="21" t="str">
         <f>IF(U446="Vacant","Vacant","")</f>
@@ -57909,7 +57893,7 @@
         <v>58</v>
       </c>
       <c r="Y460" s="21" t="s">
-        <v>60</v>
+        <v>1777</v>
       </c>
       <c r="Z460" s="21" t="str">
         <f>IF(U460="Vacant","Vacant","")</f>
@@ -58028,7 +58012,7 @@
         <v>58</v>
       </c>
       <c r="Y461" s="21" t="s">
-        <v>60</v>
+        <v>1777</v>
       </c>
       <c r="Z461" s="21" t="str">
         <f>IF(U461="Vacant","Vacant","")</f>
@@ -58585,7 +58569,7 @@
         <v>58</v>
       </c>
       <c r="Y466" s="21" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="Z466" s="21" t="str">
         <f>IF(U466="Vacant","Vacant","")</f>
@@ -64156,7 +64140,7 @@
         <v>58</v>
       </c>
       <c r="Y516" s="21" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="Z516" s="21" t="str">
         <f>IF(U516="Vacant","Vacant","")</f>

</xml_diff>